<commit_message>
test(e2e): finalize regression coverage and sprint 3 verification results
</commit_message>
<xml_diff>
--- a/docs/kiem-thu/SWP391_TestCase.xlsx
+++ b/docs/kiem-thu/SWP391_TestCase.xlsx
@@ -328,13 +328,13 @@
     <t>Có reconcile/refund</t>
   </si>
   <si>
-    <t>Ghi ý kiến hội viên, tạo yêu cầu hoàn</t>
+    <t>Ghi liên hệ bị 409: giữ nội dung; gửi lại thành công, tạo yêu cầu hoàn</t>
   </si>
   <si>
     <t>OVERPAID thừa 1000 VND</t>
   </si>
   <si>
-    <t>REFUND_PENDING, invoice vẫn PAID</t>
+    <t>Nội dung không mất khi lỗi; REFUND_PENDING, invoice vẫn PAID</t>
   </si>
   <si>
     <t>TC-S3-KPAY-03</t>

</xml_diff>

<commit_message>
docs: update BR/UC, demo script and test cases for lecturer feedback
</commit_message>
<xml_diff>
--- a/docs/kiem-thu/SWP391_TestCase.xlsx
+++ b/docs/kiem-thu/SWP391_TestCase.xlsx
@@ -8,13 +8,14 @@
     <sheet sheetId="2" name="TC-F1" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="TC-F2" state="visible" r:id="rId6"/>
     <sheet sheetId="4" name="TC-F3" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="TC-GOPY" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="308">
   <si>
     <t>ID</t>
   </si>
@@ -283,6 +284,9 @@
     <t>core/be/src/modules/class/membership-warning.test.js</t>
   </si>
   <si>
+    <t>Bỏ theo góp ý GV: học lớp không cần gói tự tập (xem TC-GOPY)</t>
+  </si>
+  <si>
     <t>TC-F2-EXP-02</t>
   </si>
   <si>
@@ -455,13 +459,493 @@
   </si>
   <si>
     <t>Chuỗi rỗng</t>
+  </si>
+  <si>
+    <t>TC-GY-01</t>
+  </si>
+  <si>
+    <t>Giờ học nằm trong khung giờ hoạt động</t>
+  </si>
+  <si>
+    <t>Có class.create</t>
+  </si>
+  <si>
+    <t>Tạo lớp giờ 12:30–13:30</t>
+  </si>
+  <si>
+    <t>Khung Sáng 09–13, Chiều 13–17</t>
+  </si>
+  <si>
+    <t>422 "không nằm trọn trong một khung giờ hoạt động"</t>
+  </si>
+  <si>
+    <t>core/be/tests/schedule-resources-gd1.test.js</t>
+  </si>
+  <si>
+    <t>TC-GY-02</t>
+  </si>
+  <si>
+    <t>Phòng đúng loại cho bộ môn</t>
+  </si>
+  <si>
+    <t>Loại phòng không dạy bộ môn</t>
+  </si>
+  <si>
+    <t>Tạo lớp chọn phòng đó</t>
+  </si>
+  <si>
+    <t>Bộ môn khác</t>
+  </si>
+  <si>
+    <t>422 "không dùng cho bộ môn này"</t>
+  </si>
+  <si>
+    <t>TC-GY-03</t>
+  </si>
+  <si>
+    <t>HLV đúng chuyên môn</t>
+  </si>
+  <si>
+    <t>HLV chưa có chuyên môn</t>
+  </si>
+  <si>
+    <t>Tạo lớp → khai báo chuyên môn → tạo lại</t>
+  </si>
+  <si>
+    <t>PUT /users/:id/subjects</t>
+  </si>
+  <si>
+    <t>422 rồi 201; không bỏ chuyên môn khi còn dạy</t>
+  </si>
+  <si>
+    <t>TC-GY-04</t>
+  </si>
+  <si>
+    <t>Xem trước khi sửa lớp</t>
+  </si>
+  <si>
+    <t>Lớp có buổi tương lai</t>
+  </si>
+  <si>
+    <t>POST /classes/:id/update-preview</t>
+  </si>
+  <si>
+    <t>Đổi giờ 20:00 → 21:00</t>
+  </si>
+  <si>
+    <t>Trả số buổi hủy/thêm, học viên, trùng lịch</t>
+  </si>
+  <si>
+    <t>TC-GY-05</t>
+  </si>
+  <si>
+    <t>Mua khóa online giữ chỗ</t>
+  </si>
+  <si>
+    <t>Lớp học phí 1.200.000, sức chứa 1</t>
+  </si>
+  <si>
+    <t>Hội viên Đăng ký khóa học</t>
+  </si>
+  <si>
+    <t>Kênh ONLINE</t>
+  </si>
+  <si>
+    <t>Hóa đơn COURSE đúng giá; PENDING_PAYMENT; người khác thấy hết chỗ; bấm lại trả cùng hóa đơn</t>
+  </si>
+  <si>
+    <t>core/be/tests/gopy-gy20-course.test.js</t>
+  </si>
+  <si>
+    <t>TC-GY-06</t>
+  </si>
+  <si>
+    <t>Hết hạn thanh toán nhả chỗ</t>
+  </si>
+  <si>
+    <t>Đang giữ chỗ</t>
+  </si>
+  <si>
+    <t>Job hết hạn hóa đơn chạy</t>
+  </si>
+  <si>
+    <t>expiresAt đã qua</t>
+  </si>
+  <si>
+    <t>Hóa đơn FAILED, đăng ký CANCELLED, mời người chờ</t>
+  </si>
+  <si>
+    <t>TC-GY-07</t>
+  </si>
+  <si>
+    <t>Thu học phí tại quầy</t>
+  </si>
+  <si>
+    <t>Lễ tân bán khóa</t>
+  </si>
+  <si>
+    <t>Tạo hóa đơn tại quầy → thu tiền mặt</t>
+  </si>
+  <si>
+    <t>memberId hội viên</t>
+  </si>
+  <si>
+    <t>Hóa đơn PAID, đăng ký BOOKED</t>
+  </si>
+  <si>
+    <t>TC-GY-08</t>
+  </si>
+  <si>
+    <t>Check-in theo khung giờ/khu vực</t>
+  </si>
+  <si>
+    <t>Gói chỉ khung khác giờ hiện tại, khu tự tập riêng</t>
+  </si>
+  <si>
+    <t>Check-in; bỏ khung; chọn sai khu; chọn đúng khu</t>
+  </si>
+  <si>
+    <t>POST /check-ins (roomTypeId)</t>
+  </si>
+  <si>
+    <t>422 "Ngoài khung giờ…", 422 "Gói không cho vào khu vực…", 201</t>
+  </si>
+  <si>
+    <t>TC-GY-09</t>
+  </si>
+  <si>
+    <t>Kỳ gói theo hóa đơn</t>
+  </si>
+  <si>
+    <t>Đang có kỳ chạy</t>
+  </si>
+  <si>
+    <t>Mua thêm gói</t>
+  </si>
+  <si>
+    <t>Thu tiền mặt / webhook</t>
+  </si>
+  <si>
+    <t>Kỳ mới nối sau kỳ cũ; /memberships/me/current có nextPeriods</t>
+  </si>
+  <si>
+    <t>core/be/tests/gopy-gy20-course.test.js; core/be/tests/sepay-webhook.test.js</t>
+  </si>
+  <si>
+    <t>TC-GY-10</t>
+  </si>
+  <si>
+    <t>Công thức hủy khóa</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>Tính cancelQuote</t>
+  </si>
+  <si>
+    <t>1.200.000 đ, 18 buổi, học 6</t>
+  </si>
+  <si>
+    <t>Còn 800.000, phí 80.000, hoàn 720.000; đổi sang khóa 1.500.000 chênh +700.000</t>
+  </si>
+  <si>
+    <t>core/be/tests/gopy-gy32-cancel-credit.test.js</t>
+  </si>
+  <si>
+    <t>TC-GY-11</t>
+  </si>
+  <si>
+    <t>Hủy khóa giữa chừng ghi số dư</t>
+  </si>
+  <si>
+    <t>Đã trả khóa, học 1/3</t>
+  </si>
+  <si>
+    <t>Xem trước → Hủy, chọn Ghi số dư</t>
+  </si>
+  <si>
+    <t>settlement CREDIT</t>
+  </si>
+  <si>
+    <t>Preview đúng công thức; số dư = số được hoàn; đăng ký CANCELLED</t>
+  </si>
+  <si>
+    <t>TC-GY-12</t>
+  </si>
+  <si>
+    <t>Dùng số dư thanh toán</t>
+  </si>
+  <si>
+    <t>Có số dư</t>
+  </si>
+  <si>
+    <t>Mua gói online → Dùng số dư</t>
+  </si>
+  <si>
+    <t>POST /invoices/:id/apply-credit</t>
+  </si>
+  <si>
+    <t>Hóa đơn PAID, kỳ gói tạo, số dư giảm đúng</t>
+  </si>
+  <si>
+    <t>TC-GY-13</t>
+  </si>
+  <si>
+    <t>Hủy kỳ chưa bắt đầu</t>
+  </si>
+  <si>
+    <t>Kỳ mua nối tiếp</t>
+  </si>
+  <si>
+    <t>Hủy, chọn Hoàn tiền</t>
+  </si>
+  <si>
+    <t>settlement REFUND</t>
+  </si>
+  <si>
+    <t>Phí 0, hoàn 100%, yêu cầu hoàn PENDING, kỳ CANCELLED</t>
+  </si>
+  <si>
+    <t>TC-GY-14</t>
+  </si>
+  <si>
+    <t>Không hủy kỳ của người khác</t>
+  </si>
+  <si>
+    <t>Token hội viên khác</t>
+  </si>
+  <si>
+    <t>GET cancel-preview</t>
+  </si>
+  <si>
+    <t>TC-GY-15</t>
+  </si>
+  <si>
+    <t>Đổi lên gói đắt hơn</t>
+  </si>
+  <si>
+    <t>Kỳ đang chạy</t>
+  </si>
+  <si>
+    <t>Xem trước → Đổi (lễ tân)</t>
+  </si>
+  <si>
+    <t>Gói 300.000 → 600.000</t>
+  </si>
+  <si>
+    <t>Hóa đơn chênh lệch tại quầy; đổi lần 2 bị 409; thu tiền → kỳ mới, kỳ cũ CANCELLED, DONE</t>
+  </si>
+  <si>
+    <t>core/be/tests/gopy-gy35-change.test.js</t>
+  </si>
+  <si>
+    <t>TC-GY-16</t>
+  </si>
+  <si>
+    <t>Đổi xuống gói rẻ hơn</t>
+  </si>
+  <si>
+    <t>Đổi không chọn cách nhận / chọn Ghi số dư</t>
+  </si>
+  <si>
+    <t>600.000 → 300.000</t>
+  </si>
+  <si>
+    <t>422 khi thiếu lựa chọn; DONE ngay, số dư = phần dư</t>
+  </si>
+  <si>
+    <t>TC-GY-17</t>
+  </si>
+  <si>
+    <t>Đổi lớp sang khóa rẻ hơn</t>
+  </si>
+  <si>
+    <t>Đã trả khóa 1.500.000</t>
+  </si>
+  <si>
+    <t>Đổi sang lớp 900.000, chọn Hoàn tiền</t>
+  </si>
+  <si>
+    <t>POST /enrollments/:id/change</t>
+  </si>
+  <si>
+    <t>Chênh −600.000, yêu cầu hoàn 600.000, lớp mới BOOKED, lớp cũ CANCELLED</t>
+  </si>
+  <si>
+    <t>TC-GY-18</t>
+  </si>
+  <si>
+    <t>Báo nghỉ trước hạn</t>
+  </si>
+  <si>
+    <t>Đã đăng ký lớp</t>
+  </si>
+  <si>
+    <t>Báo nghỉ → HLV ghi vắng sau buổi</t>
+  </si>
+  <si>
+    <t>POST /classes/sessions/:id/excuse</t>
+  </si>
+  <si>
+    <t>EXCUSED; ghi vắng không ghi đè</t>
+  </si>
+  <si>
+    <t>core/be/tests/gopy-gy30-40.test.js</t>
+  </si>
+  <si>
+    <t>TC-GY-19</t>
+  </si>
+  <si>
+    <t>Báo nghỉ quá hạn</t>
+  </si>
+  <si>
+    <t>Buổi còn &lt; 12 giờ</t>
+  </si>
+  <si>
+    <t>Báo nghỉ</t>
+  </si>
+  <si>
+    <t>422 "quá hạn báo nghỉ"</t>
+  </si>
+  <si>
+    <t>TC-GY-20</t>
+  </si>
+  <si>
+    <t>Ngân sách bảo lưu 60 ngày</t>
+  </si>
+  <si>
+    <t>Đã dùng 50 ngày</t>
+  </si>
+  <si>
+    <t>Bảo lưu 11 ngày; rồi 10 ngày</t>
+  </si>
+  <si>
+    <t>POST /memberships/:id/freezes</t>
+  </si>
+  <si>
+    <t>422; 201; chi tiết kỳ báo used 50 / left 10</t>
+  </si>
+  <si>
+    <t>TC-GY-21</t>
+  </si>
+  <si>
+    <t>Tự mở lại bảo lưu</t>
+  </si>
+  <si>
+    <t>Kỳ FROZEN, bảo lưu đã hết hạn</t>
+  </si>
+  <si>
+    <t>Job vòng đời gói chạy</t>
+  </si>
+  <si>
+    <t>9 ngày bảo lưu</t>
+  </si>
+  <si>
+    <t>Kỳ ACTIVE, cộng 9 ngày, báo hội viên một lần</t>
+  </si>
+  <si>
+    <t>TC-GY-22</t>
+  </si>
+  <si>
+    <t>Trung tâm hủy buổi bù số dư</t>
+  </si>
+  <si>
+    <t>Hội viên đã trả khóa</t>
+  </si>
+  <si>
+    <t>Quản lý hủy một buổi</t>
+  </si>
+  <si>
+    <t>Học phí 1.200.000</t>
+  </si>
+  <si>
+    <t>Số dư + giá trị một buổi (làm tròn nghìn)</t>
+  </si>
+  <si>
+    <t>TC-GY-23</t>
+  </si>
+  <si>
+    <t>Bảo lưu chặn check-in, không chặn lớp</t>
+  </si>
+  <si>
+    <t>Kỳ đang bảo lưu</t>
+  </si>
+  <si>
+    <t>Check-in; đăng ký lớp miễn phí</t>
+  </si>
+  <si>
+    <t>Check-in 422; đăng ký lớp 201; kỳ FROZEN</t>
+  </si>
+  <si>
+    <t>core/be/tests/sprint3-bao-freeze.test.js</t>
+  </si>
+  <si>
+    <t>TC-GY-24</t>
+  </si>
+  <si>
+    <t>Lớp có học phí không đăng ký miễn phí</t>
+  </si>
+  <si>
+    <t>Lớp price &gt; 0</t>
+  </si>
+  <si>
+    <t>POST /classes/:id/enrollments/me</t>
+  </si>
+  <si>
+    <t>422 "Lớp có học phí, hãy đăng ký khóa học"</t>
+  </si>
+  <si>
+    <t>core/be/tests/sprint2-class-rules.test.js</t>
+  </si>
+  <si>
+    <t>TC-GY-25</t>
+  </si>
+  <si>
+    <t>Giao diện báo nghỉ, hủy/đổi, số dư, bảo lưu (FE Khôi)</t>
+  </si>
+  <si>
+    <t>API mô phỏng</t>
+  </si>
+  <si>
+    <t>Playwright 15 ca</t>
+  </si>
+  <si>
+    <t>tests/e2e/gopy-gy36.config.mjs</t>
+  </si>
+  <si>
+    <t>Pass (bằng chứng: docs/kiem-thu/gopy-khoi-2026-10-21)</t>
+  </si>
+  <si>
+    <t>tests/e2e/gopy-gy36-contract.spec.mjs</t>
+  </si>
+  <si>
+    <t>TC-GY-26</t>
+  </si>
+  <si>
+    <t>Live E2E: mua khóa → giữ chỗ → dùng số dư → hủy ghi số dư</t>
+  </si>
+  <si>
+    <t>Lớp học phí, hội viên có số dư</t>
+  </si>
+  <si>
+    <t>Playwright với API/DB thật</t>
+  </si>
+  <si>
+    <t>gopy-gd2-4.spec.mjs</t>
+  </si>
+  <si>
+    <t>Hóa đơn khóa học, PENDING_PAYMENT → BOOKED; hủy trước ngày học hoàn 100% vào số dư</t>
+  </si>
+  <si>
+    <t>tests/e2e/gopy-gd2-4.spec.mjs</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -472,6 +956,9 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <b/>
     </font>
   </fonts>
   <fills count="3">
@@ -499,12 +986,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1316,33 +1807,33 @@
         <v>88</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>15</v>
+        <v>89</v>
       </c>
     </row>
     <row r="7" ht="54" customHeight="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>85</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>88</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>15</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -1395,25 +1886,25 @@
     </row>
     <row r="2" ht="54" customHeight="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>15</v>
@@ -1421,25 +1912,25 @@
     </row>
     <row r="3" ht="54" customHeight="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>100</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>15</v>
@@ -1447,25 +1938,25 @@
     </row>
     <row r="4" ht="54" customHeight="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>15</v>
@@ -1473,22 +1964,22 @@
     </row>
     <row r="5" ht="54" customHeight="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>51</v>
@@ -1499,22 +1990,22 @@
     </row>
     <row r="6" ht="54" customHeight="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>27</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>51</v>
@@ -1525,22 +2016,22 @@
     </row>
     <row r="7" ht="54" customHeight="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>51</v>
@@ -1551,22 +2042,22 @@
     </row>
     <row r="8" ht="54" customHeight="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>51</v>
@@ -1577,25 +2068,25 @@
     </row>
     <row r="9" ht="54" customHeight="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>15</v>
@@ -1603,25 +2094,25 @@
     </row>
     <row r="10" ht="54" customHeight="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>142</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>141</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>15</v>
@@ -1632,4 +2123,727 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H27"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="12" style="2" customWidth="1"/>
+    <col min="2" max="2" width="30" style="2" customWidth="1"/>
+    <col min="3" max="3" width="26" style="2" customWidth="1"/>
+    <col min="4" max="4" width="32" style="2" customWidth="1"/>
+    <col min="5" max="5" width="26" style="2" customWidth="1"/>
+    <col min="6" max="6" width="44" style="2" customWidth="1"/>
+    <col min="7" max="7" width="34" style="2" customWidth="1"/>
+    <col min="8" max="8" width="10" style="2" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(sprint4): deliver Khoi profile tasks and verification evidence
</commit_message>
<xml_diff>
--- a/docs/kiem-thu/SWP391_TestCase.xlsx
+++ b/docs/kiem-thu/SWP391_TestCase.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="359">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="696" uniqueCount="393">
   <si>
     <t>ID</t>
   </si>
@@ -1093,6 +1093,108 @@
   </si>
   <si>
     <t>tests/e2e/sprint4-reports.spec.mjs</t>
+  </si>
+  <si>
+    <t>TC-S4-KHOI-01</t>
+  </si>
+  <si>
+    <t>Email công khai độc lập, giới hạn giới thiệu từ cấu hình, từ chối sửa sai quyền</t>
+  </si>
+  <si>
+    <t>Migration/seed Sprint 4; fixture lớp và quyền riêng</t>
+  </si>
+  <si>
+    <t>Chạy bài kiểm thử tương ứng; E2E chạy cả desktop và mobile 320px</t>
+  </si>
+  <si>
+    <t>Dữ liệu test riêng, tự dọn sau chạy</t>
+  </si>
+  <si>
+    <t>Đúng quyền, đúng phạm vi, đồng ý chia sẻ được áp dụng tại API</t>
+  </si>
+  <si>
+    <t>core/be/tests/sprint4-coach-profile.test.js</t>
+  </si>
+  <si>
+    <t>TC-S4-KHOI-02</t>
+  </si>
+  <si>
+    <t>Danh mục HLV tìm tên/bộ môn, không lộ role/email đăng nhập/liên hệ chưa chia sẻ</t>
+  </si>
+  <si>
+    <t>TC-S4-KHOI-03</t>
+  </si>
+  <si>
+    <t>Ảnh JPG/PNG tối đa 2 MB, kiểm tra định dạng, tải có JWT và audit không chứa blob</t>
+  </si>
+  <si>
+    <t>TC-S4-KHOI-04</t>
+  </si>
+  <si>
+    <t>Hồ sơ HLV trả điểm trung bình, nhận xét ẩn danh, HLV bị khoá trả 404</t>
+  </si>
+  <si>
+    <t>TC-S4-KHOI-05</t>
+  </si>
+  <si>
+    <t>Chính chủ và nhân viên sửa hộ; từ chối giả userId và người khác không có quyền</t>
+  </si>
+  <si>
+    <t>core/be/tests/sprint4-member-profile.test.js</t>
+  </si>
+  <si>
+    <t>TC-S4-KHOI-06</t>
+  </si>
+  <si>
+    <t>HLV ngoài phân công trả 403; tắt chia sẻ không có sức khoẻ hay dữ liệu tài chính</t>
+  </si>
+  <si>
+    <t>TC-S4-KHOI-07</t>
+  </si>
+  <si>
+    <t>Được xem học viên đã học còn trong hạn, hết hạn cấu hình trả 403</t>
+  </si>
+  <si>
+    <t>TC-S4-KHOI-08</t>
+  </si>
+  <si>
+    <t>E2E desktop/mobile: HLV lưu giới thiệu/ảnh/liên hệ, giữ bản nháp khi tải ảnh</t>
+  </si>
+  <si>
+    <t>tests/e2e/sprint4-profiles.spec.mjs</t>
+  </si>
+  <si>
+    <t>TC-S4-KHOI-09</t>
+  </si>
+  <si>
+    <t>E2E desktop/mobile: tìm HLV, mở hồ sơ và deep link tới đúng lớp</t>
+  </si>
+  <si>
+    <t>TC-S4-KHOI-10</t>
+  </si>
+  <si>
+    <t>E2E desktop/mobile: bật/tắt chia sẻ, xem học viên, sửa hộ tại quầy có audit</t>
+  </si>
+  <si>
+    <t>TC-S4-KHOI-11</t>
+  </si>
+  <si>
+    <t>Ngày sinh đầu ngày Việt Nam hợp lệ khi UTC còn ngày trước</t>
+  </si>
+  <si>
+    <t>Đồng hồ test 00:30 Việt Nam</t>
+  </si>
+  <si>
+    <t>Kiểm tra hôm nay, ngày mai và giá trị bỏ trống</t>
+  </si>
+  <si>
+    <t>2026-10-28T17:30Z; ngày sinh 29/10, 30/10 và null</t>
+  </si>
+  <si>
+    <t>Nhận ngày hôm nay/null, từ chối ngày mai</t>
+  </si>
+  <si>
+    <t>core/be/src/modules/profile/profile.validation.test.js</t>
   </si>
 </sst>
 </file>
@@ -3013,7 +3115,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" style="2" customWidth="1"/>
@@ -3598,8 +3700,294 @@
         <v>15</v>
       </c>
     </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>